<commit_message>
Implement RVV integer extension ALU forms
</commit_message>
<xml_diff>
--- a/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
+++ b/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="R359ca7c0b84c4f8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="Rdd29b7e7e51a45af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="Rae7af9e3bb174289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R664ac2cd04914964"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="Re4b9b93f87ec4967"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R9eb5c0f70d3b4eab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R04917c95e9ac4b34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R9d2cb415bb454313"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35840,7 +35840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c691d1202de4096"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1d10523972e4f29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36328,20 +36328,20 @@
       </x:c>
       <x:c r="B2" s="18" t="n">
         <x:f>COUNTIF(I6:I285,"yes")</x:f>
-        <x:v>159</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
         <x:v>실행</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
         <x:f>COUNTIF(J6:J285,"yes")</x:f>
-        <x:v>159</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
         <x:v>TOP 테스트</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
-        <x:v>12</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
         <x:v>전체</x:v>
@@ -45070,13 +45070,17 @@
         <x:v>b00111</x:v>
       </x:c>
       <x:c r="I251" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J251" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K251" s="20" t="str"/>
-      <x:c r="L251" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K251" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L251" s="20" t="str">
+        <x:v>signed halfword lanes; fractional overlap rejection</x:v>
+      </x:c>
       <x:c r="M251" s="20" t="str"/>
     </x:row>
     <x:row r="252" ht="19" customHeight="1">
@@ -45105,13 +45109,17 @@
         <x:v>b00101</x:v>
       </x:c>
       <x:c r="I252" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J252" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K252" s="20" t="str"/>
-      <x:c r="L252" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K252" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L252" s="20" t="str">
+        <x:v>m4, signed byte lanes</x:v>
+      </x:c>
       <x:c r="M252" s="20" t="str"/>
     </x:row>
     <x:row r="253" ht="19" customHeight="1">
@@ -45140,13 +45148,17 @@
         <x:v>b00011</x:v>
       </x:c>
       <x:c r="I253" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J253" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K253" s="20" t="str"/>
-      <x:c r="L253" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K253" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L253" s="20" t="str">
+        <x:v>signed byte lanes at SEW=64</x:v>
+      </x:c>
       <x:c r="M253" s="20" t="str"/>
     </x:row>
     <x:row r="254" ht="19" customHeight="1">
@@ -46190,13 +46202,17 @@
         <x:v>b00110</x:v>
       </x:c>
       <x:c r="I283" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J283" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K283" s="20" t="str"/>
-      <x:c r="L283" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K283" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L283" s="20" t="str">
+        <x:v>m2, shared source register across beats</x:v>
+      </x:c>
       <x:c r="M283" s="20" t="str"/>
     </x:row>
     <x:row r="284" ht="19" customHeight="1">
@@ -46225,13 +46241,17 @@
         <x:v>b00100</x:v>
       </x:c>
       <x:c r="I284" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J284" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K284" s="20" t="str"/>
-      <x:c r="L284" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K284" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L284" s="20" t="str">
+        <x:v>byte zero extension</x:v>
+      </x:c>
       <x:c r="M284" s="20" t="str"/>
     </x:row>
     <x:row r="285" ht="19" customHeight="1">
@@ -46260,19 +46280,23 @@
         <x:v>b00010</x:v>
       </x:c>
       <x:c r="I285" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J285" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K285" s="20" t="str"/>
-      <x:c r="L285" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K285" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L285" s="20" t="str">
+        <x:v>m8, source EMUL=1; overlap boundary</x:v>
+      </x:c>
       <x:c r="M285" s="20" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47114c8551854620"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92b12db18cad434a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add RVV widening integer add and subtract
</commit_message>
<xml_diff>
--- a/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
+++ b/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="Re4b9b93f87ec4967"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R9eb5c0f70d3b4eab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R04917c95e9ac4b34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R9d2cb415bb454313"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="R5b098179c1f1436d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R42dec6659dd14b4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R38b8d8c6d60e4abc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R9b37b6c5f7104d46"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35840,7 +35840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1d10523972e4f29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb326cd3f10ec47d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36328,20 +36328,20 @@
       </x:c>
       <x:c r="B2" s="18" t="n">
         <x:f>COUNTIF(I6:I285,"yes")</x:f>
-        <x:v>165</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
         <x:v>실행</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
         <x:f>COUNTIF(J6:J285,"yes")</x:f>
-        <x:v>165</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
         <x:v>TOP 테스트</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
-        <x:v>18</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
         <x:v>전체</x:v>
@@ -45187,13 +45187,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I254" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J254" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K254" s="20" t="str"/>
-      <x:c r="L254" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K254" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L254" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M254" s="20" t="str"/>
     </x:row>
     <x:row r="255" ht="19" customHeight="1">
@@ -45222,13 +45226,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I255" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J255" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K255" s="20" t="str"/>
-      <x:c r="L255" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K255" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L255" s="20" t="str">
+        <x:v>signed scalar widened; negative lanes</x:v>
+      </x:c>
       <x:c r="M255" s="20" t="str"/>
     </x:row>
     <x:row r="256" ht="19" customHeight="1">
@@ -45257,13 +45265,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I256" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J256" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K256" s="20" t="str"/>
-      <x:c r="L256" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K256" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L256" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M256" s="20" t="str"/>
     </x:row>
     <x:row r="257" ht="19" customHeight="1">
@@ -45292,13 +45304,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I257" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J257" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K257" s="20" t="str"/>
-      <x:c r="L257" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K257" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L257" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M257" s="20" t="str"/>
     </x:row>
     <x:row r="258" ht="19" customHeight="1">
@@ -45327,13 +45343,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I258" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J258" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K258" s="20" t="str"/>
-      <x:c r="L258" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K258" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L258" s="20" t="str">
+        <x:v>m2 source, m4 destination</x:v>
+      </x:c>
       <x:c r="M258" s="20" t="str"/>
     </x:row>
     <x:row r="259" ht="19" customHeight="1">
@@ -45362,13 +45382,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I259" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J259" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K259" s="20" t="str"/>
-      <x:c r="L259" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K259" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L259" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M259" s="20" t="str"/>
     </x:row>
     <x:row r="260" ht="19" customHeight="1">
@@ -45397,13 +45421,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I260" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J260" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K260" s="20" t="str"/>
-      <x:c r="L260" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K260" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L260" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M260" s="20" t="str"/>
     </x:row>
     <x:row r="261" ht="19" customHeight="1">
@@ -45432,13 +45460,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I261" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J261" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K261" s="20" t="str"/>
-      <x:c r="L261" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K261" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L261" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M261" s="20" t="str"/>
     </x:row>
     <x:row r="262" ht="19" customHeight="1">
@@ -45922,13 +45954,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I275" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J275" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K275" s="20" t="str"/>
-      <x:c r="L275" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K275" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L275" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M275" s="20" t="str"/>
     </x:row>
     <x:row r="276" ht="19" customHeight="1">
@@ -45957,13 +45993,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I276" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J276" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K276" s="20" t="str"/>
-      <x:c r="L276" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K276" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L276" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M276" s="20" t="str"/>
     </x:row>
     <x:row r="277" ht="19" customHeight="1">
@@ -45992,13 +46032,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I277" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J277" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K277" s="20" t="str"/>
-      <x:c r="L277" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K277" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L277" s="20" t="str">
+        <x:v>wide vs2, narrow vs1; destructive vd</x:v>
+      </x:c>
       <x:c r="M277" s="20" t="str"/>
     </x:row>
     <x:row r="278" ht="19" customHeight="1">
@@ -46027,13 +46071,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I278" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J278" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K278" s="20" t="str"/>
-      <x:c r="L278" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K278" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L278" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M278" s="20" t="str"/>
     </x:row>
     <x:row r="279" ht="19" customHeight="1">
@@ -46062,13 +46110,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I279" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J279" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K279" s="20" t="str"/>
-      <x:c r="L279" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K279" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L279" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M279" s="20" t="str"/>
     </x:row>
     <x:row r="280" ht="19" customHeight="1">
@@ -46097,13 +46149,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I280" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J280" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K280" s="20" t="str"/>
-      <x:c r="L280" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K280" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L280" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M280" s="20" t="str"/>
     </x:row>
     <x:row r="281" ht="19" customHeight="1">
@@ -46132,13 +46188,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I281" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J281" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K281" s="20" t="str"/>
-      <x:c r="L281" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K281" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L281" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M281" s="20" t="str"/>
     </x:row>
     <x:row r="282" ht="19" customHeight="1">
@@ -46167,13 +46227,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I282" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J282" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K282" s="20" t="str"/>
-      <x:c r="L282" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K282" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L282" s="20" t="str">
+        <x:v>m1 all lanes, OP-MVV/OP-MVX sweep</x:v>
+      </x:c>
       <x:c r="M282" s="20" t="str"/>
     </x:row>
     <x:row r="283" ht="19" customHeight="1">
@@ -46296,7 +46360,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92b12db18cad434a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd5522395648404d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add RVV widening integer multiply and MAC
</commit_message>
<xml_diff>
--- a/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
+++ b/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="R5b098179c1f1436d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R42dec6659dd14b4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R38b8d8c6d60e4abc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R9b37b6c5f7104d46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="Ra94c0f5de6094680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R5285c6045fec4e31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R64765f71c5c04aa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="Rd4c82444f4ef44af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35840,7 +35840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb326cd3f10ec47d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ee476e7ab1843e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36328,20 +36328,20 @@
       </x:c>
       <x:c r="B2" s="18" t="n">
         <x:f>COUNTIF(I6:I285,"yes")</x:f>
-        <x:v>181</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
         <x:v>실행</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
         <x:f>COUNTIF(J6:J285,"yes")</x:f>
-        <x:v>181</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
         <x:v>TOP 테스트</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
-        <x:v>34</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
         <x:v>전체</x:v>
@@ -45499,13 +45499,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I262" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J262" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K262" s="20" t="str"/>
-      <x:c r="L262" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K262" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L262" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M262" s="20" t="str"/>
     </x:row>
     <x:row r="263" ht="19" customHeight="1">
@@ -45534,13 +45538,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I263" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J263" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K263" s="20" t="str"/>
-      <x:c r="L263" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K263" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L263" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M263" s="20" t="str"/>
     </x:row>
     <x:row r="264" ht="19" customHeight="1">
@@ -45569,13 +45577,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I264" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J264" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K264" s="20" t="str"/>
-      <x:c r="L264" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K264" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L264" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M264" s="20" t="str"/>
     </x:row>
     <x:row r="265" ht="19" customHeight="1">
@@ -45604,13 +45616,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I265" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J265" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K265" s="20" t="str"/>
-      <x:c r="L265" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K265" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L265" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M265" s="20" t="str"/>
     </x:row>
     <x:row r="266" ht="19" customHeight="1">
@@ -45639,13 +45655,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I266" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J266" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K266" s="20" t="str"/>
-      <x:c r="L266" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K266" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L266" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M266" s="20" t="str"/>
     </x:row>
     <x:row r="267" ht="19" customHeight="1">
@@ -45674,13 +45694,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I267" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J267" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K267" s="20" t="str"/>
-      <x:c r="L267" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K267" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L267" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M267" s="20" t="str"/>
     </x:row>
     <x:row r="268" ht="19" customHeight="1">
@@ -45709,13 +45733,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I268" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J268" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K268" s="20" t="str"/>
-      <x:c r="L268" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K268" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L268" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M268" s="20" t="str"/>
     </x:row>
     <x:row r="269" ht="19" customHeight="1">
@@ -45744,13 +45772,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I269" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J269" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K269" s="20" t="str"/>
-      <x:c r="L269" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K269" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L269" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M269" s="20" t="str"/>
     </x:row>
     <x:row r="270" ht="19" customHeight="1">
@@ -45779,13 +45811,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I270" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J270" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K270" s="20" t="str"/>
-      <x:c r="L270" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K270" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L270" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M270" s="20" t="str"/>
     </x:row>
     <x:row r="271" ht="19" customHeight="1">
@@ -45814,13 +45850,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I271" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J271" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K271" s="20" t="str"/>
-      <x:c r="L271" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K271" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L271" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M271" s="20" t="str"/>
     </x:row>
     <x:row r="272" ht="19" customHeight="1">
@@ -45849,13 +45889,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I272" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J272" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K272" s="20" t="str"/>
-      <x:c r="L272" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K272" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L272" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M272" s="20" t="str"/>
     </x:row>
     <x:row r="273" ht="19" customHeight="1">
@@ -45884,13 +45928,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I273" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J273" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K273" s="20" t="str"/>
-      <x:c r="L273" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K273" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L273" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M273" s="20" t="str"/>
     </x:row>
     <x:row r="274" ht="19" customHeight="1">
@@ -45919,13 +45967,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I274" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J274" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K274" s="20" t="str"/>
-      <x:c r="L274" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K274" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L274" s="20" t="str">
+        <x:v>m1 all lanes; signed/unsigned corners; MAC old vd</x:v>
+      </x:c>
       <x:c r="M274" s="20" t="str"/>
     </x:row>
     <x:row r="275" ht="19" customHeight="1">
@@ -46360,7 +46412,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd5522395648404d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R928f56ad0be64172"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implement RVV narrowing shifts and clips in ALU
</commit_message>
<xml_diff>
--- a/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
+++ b/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="Ra94c0f5de6094680"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R5285c6045fec4e31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R64765f71c5c04aa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="Rd4c82444f4ef44af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="R79fa40e772ec4911"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R1513e1701c174289"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R81fd1739e10e4274"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R425e205a39ad4aa3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35840,7 +35840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ee476e7ab1843e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re09bbd68a62b4cd8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36328,20 +36328,20 @@
       </x:c>
       <x:c r="B2" s="18" t="n">
         <x:f>COUNTIF(I6:I285,"yes")</x:f>
-        <x:v>194</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
         <x:v>실행</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
         <x:f>COUNTIF(J6:J285,"yes")</x:f>
-        <x:v>194</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
         <x:v>TOP 테스트</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
-        <x:v>47</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
         <x:v>전체</x:v>
@@ -44650,13 +44650,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I239" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J239" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K239" s="20" t="str"/>
-      <x:c r="L239" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K239" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L239" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M239" s="20" t="str"/>
     </x:row>
     <x:row r="240" ht="19" customHeight="1">
@@ -44685,13 +44689,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I240" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J240" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K240" s="20" t="str"/>
-      <x:c r="L240" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K240" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L240" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M240" s="20" t="str"/>
     </x:row>
     <x:row r="241" ht="19" customHeight="1">
@@ -44720,13 +44728,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I241" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J241" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K241" s="20" t="str"/>
-      <x:c r="L241" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K241" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L241" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M241" s="20" t="str"/>
     </x:row>
     <x:row r="242" ht="19" customHeight="1">
@@ -44755,13 +44767,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I242" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J242" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K242" s="20" t="str"/>
-      <x:c r="L242" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K242" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L242" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M242" s="20" t="str"/>
     </x:row>
     <x:row r="243" ht="19" customHeight="1">
@@ -44790,13 +44806,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I243" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J243" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K243" s="20" t="str"/>
-      <x:c r="L243" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K243" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L243" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M243" s="20" t="str"/>
     </x:row>
     <x:row r="244" ht="19" customHeight="1">
@@ -44825,13 +44845,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I244" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J244" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K244" s="20" t="str"/>
-      <x:c r="L244" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K244" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L244" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M244" s="20" t="str"/>
     </x:row>
     <x:row r="245" ht="19" customHeight="1">
@@ -44860,13 +44884,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I245" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J245" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K245" s="20" t="str"/>
-      <x:c r="L245" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K245" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L245" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M245" s="20" t="str"/>
     </x:row>
     <x:row r="246" ht="19" customHeight="1">
@@ -44895,13 +44923,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I246" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J246" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K246" s="20" t="str"/>
-      <x:c r="L246" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K246" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L246" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M246" s="20" t="str"/>
     </x:row>
     <x:row r="247" ht="19" customHeight="1">
@@ -44930,13 +44962,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I247" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J247" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K247" s="20" t="str"/>
-      <x:c r="L247" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K247" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L247" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M247" s="20" t="str"/>
     </x:row>
     <x:row r="248" ht="19" customHeight="1">
@@ -44965,13 +45001,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I248" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J248" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K248" s="20" t="str"/>
-      <x:c r="L248" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K248" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L248" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M248" s="20" t="str"/>
     </x:row>
     <x:row r="249" ht="19" customHeight="1">
@@ -45000,13 +45040,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I249" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J249" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K249" s="20" t="str"/>
-      <x:c r="L249" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K249" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L249" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M249" s="20" t="str"/>
     </x:row>
     <x:row r="250" ht="19" customHeight="1">
@@ -45035,13 +45079,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I250" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J250" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K250" s="20" t="str"/>
-      <x:c r="L250" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K250" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L250" s="20" t="str">
+        <x:v>1R wide source pair, m2/mf2, overlap, vxrm, masked vxsat</x:v>
+      </x:c>
       <x:c r="M250" s="20" t="str"/>
     </x:row>
     <x:row r="251" ht="19" customHeight="1">
@@ -46412,7 +46460,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R928f56ad0be64172"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ccb705b4bdc4cfa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add FP32 min and max vector reductions
</commit_message>
<xml_diff>
--- a/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
+++ b/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="R79fa40e772ec4911"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R1513e1701c174289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R81fd1739e10e4274"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R425e205a39ad4aa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="Ra402e5f830a94bac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R2c18fe56ae304575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R45dcf5c78a804fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R7f89b32d8b384455"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35840,7 +35840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re09bbd68a62b4cd8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refa888a312374a6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36328,20 +36328,20 @@
       </x:c>
       <x:c r="B2" s="18" t="n">
         <x:f>COUNTIF(I6:I285,"yes")</x:f>
-        <x:v>206</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
         <x:v>실행</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
         <x:f>COUNTIF(J6:J285,"yes")</x:f>
-        <x:v>206</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
         <x:v>TOP 테스트</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
-        <x:v>59</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
         <x:v>전체</x:v>
@@ -40103,13 +40103,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I110" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J110" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K110" s="20" t="str"/>
-      <x:c r="L110" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K110" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L110" s="20" t="str">
+        <x:v>m2, NaN/zero, mask and fflags</x:v>
+      </x:c>
       <x:c r="M110" s="20" t="str"/>
     </x:row>
     <x:row r="111" ht="19" customHeight="1">
@@ -40138,13 +40142,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I111" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J111" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K111" s="20" t="str"/>
-      <x:c r="L111" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K111" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L111" s="20" t="str">
+        <x:v>m2, NaN/zero, mask and fflags</x:v>
+      </x:c>
       <x:c r="M111" s="20" t="str"/>
     </x:row>
     <x:row r="112" ht="19" customHeight="1">
@@ -46460,7 +46468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ccb705b4bdc4cfa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ed9b1c8452c468e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implement shared FP32 add, multiply and fused vector ALU path
</commit_message>
<xml_diff>
--- a/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
+++ b/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="Ra402e5f830a94bac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R2c18fe56ae304575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R45dcf5c78a804fc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R7f89b32d8b384455"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="R833e827173ec4fd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R6e22564c5e8444c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="Ra9e27b6213284cb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R8c84237a470a41ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35840,7 +35840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refa888a312374a6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf94c46a3e1764cda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36328,20 +36328,20 @@
       </x:c>
       <x:c r="B2" s="18" t="n">
         <x:f>COUNTIF(I6:I285,"yes")</x:f>
-        <x:v>208</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
         <x:v>실행</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
         <x:f>COUNTIF(J6:J285,"yes")</x:f>
-        <x:v>208</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
         <x:v>TOP 테스트</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
-        <x:v>61</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
         <x:v>전체</x:v>
@@ -37711,13 +37711,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I42" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J42" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K42" s="20" t="str"/>
-      <x:c r="L42" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K42" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L42" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M42" s="20" t="str"/>
     </x:row>
     <x:row r="43" ht="19" customHeight="1">
@@ -37746,13 +37750,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I43" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J43" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K43" s="20" t="str"/>
-      <x:c r="L43" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K43" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L43" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M43" s="20" t="str"/>
     </x:row>
     <x:row r="44" ht="19" customHeight="1">
@@ -37995,13 +38003,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I50" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J50" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K50" s="20" t="str"/>
-      <x:c r="L50" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K50" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L50" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M50" s="20" t="str"/>
     </x:row>
     <x:row r="51" ht="19" customHeight="1">
@@ -38279,13 +38291,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I58" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J58" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K58" s="20" t="str"/>
-      <x:c r="L58" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K58" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L58" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M58" s="20" t="str"/>
     </x:row>
     <x:row r="59" ht="19" customHeight="1">
@@ -38314,13 +38330,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I59" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J59" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K59" s="20" t="str"/>
-      <x:c r="L59" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K59" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L59" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M59" s="20" t="str"/>
     </x:row>
     <x:row r="60" ht="19" customHeight="1">
@@ -38983,13 +39003,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I78" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J78" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K78" s="20" t="str"/>
-      <x:c r="L78" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K78" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L78" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M78" s="20" t="str"/>
     </x:row>
     <x:row r="79" ht="19" customHeight="1">
@@ -39018,13 +39042,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I79" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J79" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K79" s="20" t="str"/>
-      <x:c r="L79" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K79" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L79" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M79" s="20" t="str"/>
     </x:row>
     <x:row r="80" ht="19" customHeight="1">
@@ -39053,13 +39081,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I80" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J80" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K80" s="20" t="str"/>
-      <x:c r="L80" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K80" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L80" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M80" s="20" t="str"/>
     </x:row>
     <x:row r="81" ht="19" customHeight="1">
@@ -39088,13 +39120,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I81" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J81" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K81" s="20" t="str"/>
-      <x:c r="L81" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K81" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L81" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M81" s="20" t="str"/>
     </x:row>
     <x:row r="82" ht="19" customHeight="1">
@@ -39263,13 +39299,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I86" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J86" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K86" s="20" t="str"/>
-      <x:c r="L86" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K86" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L86" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M86" s="20" t="str"/>
     </x:row>
     <x:row r="87" ht="19" customHeight="1">
@@ -39298,13 +39338,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I87" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J87" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K87" s="20" t="str"/>
-      <x:c r="L87" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K87" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L87" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M87" s="20" t="str"/>
     </x:row>
     <x:row r="88" ht="19" customHeight="1">
@@ -39333,13 +39377,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I88" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J88" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K88" s="20" t="str"/>
-      <x:c r="L88" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K88" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L88" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M88" s="20" t="str"/>
     </x:row>
     <x:row r="89" ht="19" customHeight="1">
@@ -39368,13 +39416,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I89" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J89" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K89" s="20" t="str"/>
-      <x:c r="L89" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K89" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L89" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M89" s="20" t="str"/>
     </x:row>
     <x:row r="90" ht="19" customHeight="1">
@@ -39403,13 +39455,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I90" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J90" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K90" s="20" t="str"/>
-      <x:c r="L90" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K90" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L90" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M90" s="20" t="str"/>
     </x:row>
     <x:row r="91" ht="19" customHeight="1">
@@ -39438,13 +39494,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I91" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J91" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K91" s="20" t="str"/>
-      <x:c r="L91" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K91" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L91" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M91" s="20" t="str"/>
     </x:row>
     <x:row r="92" ht="19" customHeight="1">
@@ -39473,13 +39533,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I92" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J92" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K92" s="20" t="str"/>
-      <x:c r="L92" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K92" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L92" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M92" s="20" t="str"/>
     </x:row>
     <x:row r="93" ht="19" customHeight="1">
@@ -39508,13 +39572,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I93" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J93" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K93" s="20" t="str"/>
-      <x:c r="L93" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K93" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L93" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M93" s="20" t="str"/>
     </x:row>
     <x:row r="94" ht="19" customHeight="1">
@@ -39543,13 +39611,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I94" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J94" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K94" s="20" t="str"/>
-      <x:c r="L94" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K94" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L94" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M94" s="20" t="str"/>
     </x:row>
     <x:row r="95" ht="19" customHeight="1">
@@ -39578,13 +39650,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I95" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J95" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K95" s="20" t="str"/>
-      <x:c r="L95" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K95" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L95" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M95" s="20" t="str"/>
     </x:row>
     <x:row r="96" ht="19" customHeight="1">
@@ -39613,13 +39689,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I96" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J96" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K96" s="20" t="str"/>
-      <x:c r="L96" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K96" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L96" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M96" s="20" t="str"/>
     </x:row>
     <x:row r="97" ht="19" customHeight="1">
@@ -39648,13 +39728,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I97" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J97" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K97" s="20" t="str"/>
-      <x:c r="L97" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K97" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L97" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M97" s="20" t="str"/>
     </x:row>
     <x:row r="98" ht="19" customHeight="1">
@@ -39683,13 +39767,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I98" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J98" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K98" s="20" t="str"/>
-      <x:c r="L98" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K98" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L98" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M98" s="20" t="str"/>
     </x:row>
     <x:row r="99" ht="19" customHeight="1">
@@ -39718,13 +39806,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I99" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J99" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K99" s="20" t="str"/>
-      <x:c r="L99" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K99" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L99" s="20" t="str">
+        <x:v>shared fused FP32 path; all forms, frm, NV/OF/UF/NX, m2</x:v>
+      </x:c>
       <x:c r="M99" s="20" t="str"/>
     </x:row>
     <x:row r="100" ht="19" customHeight="1">
@@ -46468,7 +46560,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ed9b1c8452c468e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R495b27e8aab04e52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete RV32IMFC vector ALU instruction profile
</commit_message>
<xml_diff>
--- a/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
+++ b/outputs/rvv_instruction_20260916/RVV_Instruction_Decode_RV32.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="R833e827173ec4fd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R6e22564c5e8444c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="Ra9e27b6213284cb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="R8c84237a470a41ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개요" sheetId="1" r:id="Re5621d52a9d9417b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명령어" sheetId="2" r:id="R1e42037f670442c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="디코드 기준" sheetId="3" r:id="R24a4884926554677"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALU 구현" sheetId="4" r:id="Rfbcfee47b8634dc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35840,7 +35840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf94c46a3e1764cda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a176a488eaa4e53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36328,20 +36328,20 @@
       </x:c>
       <x:c r="B2" s="18" t="n">
         <x:f>COUNTIF(I6:I285,"yes")</x:f>
-        <x:v>231</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="C2" s="18" t="str">
         <x:v>실행</x:v>
       </x:c>
       <x:c r="D2" s="18" t="n">
         <x:f>COUNTIF(J6:J285,"yes")</x:f>
-        <x:v>231</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="E2" s="18" t="str">
         <x:v>TOP 테스트</x:v>
       </x:c>
       <x:c r="F2" s="18" t="n">
-        <x:v>84</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="G2" s="18" t="str">
         <x:v>전체</x:v>
@@ -36976,13 +36976,17 @@
         <x:v>b00011</x:v>
       </x:c>
       <x:c r="I21" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J21" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K21" s="20" t="str"/>
-      <x:c r="L21" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K21" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L21" s="20" t="str">
+        <x:v>all four lanes; NX, signed/unsigned saturation, NaN, RTZ</x:v>
+      </x:c>
       <x:c r="M21" s="20" t="str"/>
     </x:row>
     <x:row r="22" ht="19" customHeight="1">
@@ -37011,13 +37015,17 @@
         <x:v>b00010</x:v>
       </x:c>
       <x:c r="I22" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J22" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K22" s="20" t="str"/>
-      <x:c r="L22" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K22" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L22" s="20" t="str">
+        <x:v>all four lanes; NX, signed/unsigned saturation, NaN, RTZ</x:v>
+      </x:c>
       <x:c r="M22" s="20" t="str"/>
     </x:row>
     <x:row r="23" ht="19" customHeight="1">
@@ -37046,13 +37054,17 @@
         <x:v>b00111</x:v>
       </x:c>
       <x:c r="I23" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J23" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K23" s="20" t="str"/>
-      <x:c r="L23" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K23" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L23" s="20" t="str">
+        <x:v>all four lanes; NX, signed/unsigned saturation, NaN, RTZ</x:v>
+      </x:c>
       <x:c r="M23" s="20" t="str"/>
     </x:row>
     <x:row r="24" ht="19" customHeight="1">
@@ -37081,13 +37093,17 @@
         <x:v>b00110</x:v>
       </x:c>
       <x:c r="I24" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J24" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K24" s="20" t="str"/>
-      <x:c r="L24" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K24" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L24" s="20" t="str">
+        <x:v>all four lanes; NX, signed/unsigned saturation, NaN, RTZ</x:v>
+      </x:c>
       <x:c r="M24" s="20" t="str"/>
     </x:row>
     <x:row r="25" ht="19" customHeight="1">
@@ -37116,13 +37132,17 @@
         <x:v>b00001</x:v>
       </x:c>
       <x:c r="I25" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J25" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K25" s="20" t="str"/>
-      <x:c r="L25" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K25" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L25" s="20" t="str">
+        <x:v>all four lanes; NX, signed/unsigned saturation, NaN, RTZ</x:v>
+      </x:c>
       <x:c r="M25" s="20" t="str"/>
     </x:row>
     <x:row r="26" ht="19" customHeight="1">
@@ -37151,13 +37171,17 @@
         <x:v>b00000</x:v>
       </x:c>
       <x:c r="I26" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J26" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K26" s="20" t="str"/>
-      <x:c r="L26" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K26" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L26" s="20" t="str">
+        <x:v>all four lanes; NX, signed/unsigned saturation, NaN, RTZ</x:v>
+      </x:c>
       <x:c r="M26" s="20" t="str"/>
     </x:row>
     <x:row r="27" ht="19" customHeight="1">
@@ -37828,13 +37852,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I45" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J45" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K45" s="20" t="str"/>
-      <x:c r="L45" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K45" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L45" s="20" t="str">
+        <x:v>iterative shared unit; vv/vf, DZ/NV, mask</x:v>
+      </x:c>
       <x:c r="M45" s="20" t="str"/>
     </x:row>
     <x:row r="46" ht="19" customHeight="1">
@@ -37863,13 +37891,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I46" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J46" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K46" s="20" t="str"/>
-      <x:c r="L46" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K46" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L46" s="20" t="str">
+        <x:v>iterative shared unit; vv/vf, DZ/NV, mask</x:v>
+      </x:c>
       <x:c r="M46" s="20" t="str"/>
     </x:row>
     <x:row r="47" ht="19" customHeight="1">
@@ -37898,13 +37930,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I47" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J47" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K47" s="20" t="str"/>
-      <x:c r="L47" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K47" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L47" s="20" t="str">
+        <x:v>iterative shared unit; vv/vf, DZ/NV, mask</x:v>
+      </x:c>
       <x:c r="M47" s="20" t="str"/>
     </x:row>
     <x:row r="48" ht="19" customHeight="1">
@@ -37933,13 +37969,17 @@
         <x:v>b00101</x:v>
       </x:c>
       <x:c r="I48" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J48" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K48" s="20" t="str"/>
-      <x:c r="L48" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K48" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L48" s="20" t="str">
+        <x:v>RVV 1.0 128-entry LUT; normal/subnormal examples, NV/DZ/OF/NX</x:v>
+      </x:c>
       <x:c r="M48" s="20" t="str"/>
     </x:row>
     <x:row r="49" ht="19" customHeight="1">
@@ -37968,13 +38008,17 @@
         <x:v>b00100</x:v>
       </x:c>
       <x:c r="I49" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J49" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K49" s="20" t="str"/>
-      <x:c r="L49" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K49" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L49" s="20" t="str">
+        <x:v>RVV 1.0 128-entry LUT; normal/subnormal examples, NV/DZ/OF/NX</x:v>
+      </x:c>
       <x:c r="M49" s="20" t="str"/>
     </x:row>
     <x:row r="50" ht="19" customHeight="1">
@@ -38256,13 +38300,17 @@
         <x:v>b00000</x:v>
       </x:c>
       <x:c r="I57" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J57" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K57" s="20" t="str"/>
-      <x:c r="L57" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K57" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L57" s="20" t="str">
+        <x:v>iterative shared unit; vv/vf, DZ/NV, mask</x:v>
+      </x:c>
       <x:c r="M57" s="20" t="str"/>
     </x:row>
     <x:row r="58" ht="19" customHeight="1">
@@ -40273,13 +40321,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I112" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J112" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K112" s="20" t="str"/>
-      <x:c r="L112" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K112" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L112" s="20" t="str">
+        <x:v>m2 seed carry, masked sNaN seed, ordered shared FMA</x:v>
+      </x:c>
       <x:c r="M112" s="20" t="str"/>
     </x:row>
     <x:row r="113" ht="19" customHeight="1">
@@ -40308,13 +40360,17 @@
         <x:v>variable</x:v>
       </x:c>
       <x:c r="I113" s="20" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="J113" s="20" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="K113" s="20" t="str"/>
-      <x:c r="L113" s="20" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="K113" s="20" t="str">
+        <x:v>tb_vcore_alu_top</x:v>
+      </x:c>
+      <x:c r="L113" s="20" t="str">
+        <x:v>m2 seed carry, masked sNaN seed, ordered shared FMA</x:v>
+      </x:c>
       <x:c r="M113" s="20" t="str"/>
     </x:row>
     <x:row r="114" ht="19" customHeight="1">
@@ -46560,7 +46616,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R495b27e8aab04e52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc596bcdb5dd54b5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>